<commit_message>
Align continuity plan workbook to paired review
</commit_message>
<xml_diff>
--- a/templates/if-something-happened-to-me-information-plan/information-plan.xlsx
+++ b/templates/if-something-happened-to-me-information-plan/information-plan.xlsx
@@ -11,14 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Map" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Loops" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recurring Responsibilities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protected Access" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Authority &amp; Access" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Test" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Handoff Map'!$A$4:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Handoff Map'!$A$4:$D$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Open Loops'!$A$4:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Recurring Responsibilities'!$A$4:$E$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Protected Access'!$A$4:$E$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Authority &amp; Access'!$A$4:$E$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +70,51 @@
     <font>
       <color rgb="00008000"/>
     </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="0017324D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="00C65911"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -99,7 +144,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -107,11 +152,69 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9E1F2"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9E1F2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E1F2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E1F2"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E1F2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E1F2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E1F2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E1F2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E1F2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E1F2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E1F2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E1F2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -152,6 +255,38 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -519,13 +654,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
@@ -544,7 +679,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="54" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -577,7 +711,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Who matters?  What exists?  Where does the real information live?  What is happening now?  What needs to keep happening?</t>
+          <t>Taken together, the plan answers: Who matters?  What exists?  Where does the real information live?  What is happening now?  What needs to keep happening?</t>
         </is>
       </c>
     </row>
@@ -593,7 +727,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
+    <row r="8" ht="55" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Security rule</t>
@@ -601,7 +735,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Never put passwords, PINs, recovery codes, encryption keys, banking credentials, security answers, or other secrets in this workbook.</t>
+          <t>Never put passwords, PINs, recovery codes, encryption keys, banking credentials, security answers, or other secrets in this workbook. Even without secrets, the completed plan can be sensitive; keep and share it appropriately.</t>
         </is>
       </c>
     </row>
@@ -613,14 +747,14 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Start with the few areas where another person would lose time, money, care continuity, or important context if you were unavailable for two weeks.</t>
+          <t>Write each detail once. Use the Handoff Map as an index; keep open situations, recurring responsibilities, formal authorities, and protected access in their natural sections.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="54" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Different from #6</t>
+          <t>Different from emergency checklist</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -629,12 +763,26 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Start small</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Begin with two or three people to contact, three to five household areas another person could not reconstruct, and anything open or due in the next two weeks.</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="20" t="n"/>
+    </row>
     <row r="13" ht="25" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Plan owner</t>
+          <t>Plan owner(s)</t>
         </is>
       </c>
       <c r="B13" s="6" t="n"/>
@@ -663,21 +811,120 @@
       </c>
       <c r="B16" s="6" t="n"/>
     </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>People to Contact First</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="n"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="20" t="n"/>
+    </row>
+    <row r="20" ht="35" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Add only the few people someone should contact first. This is contact information, not a grant of authority.</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="20" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="n"/>
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="21" t="n"/>
+      <c r="D21" s="21" t="n"/>
+      <c r="E21" s="21" t="n"/>
+      <c r="F21" s="21" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Person / role</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Why they matter</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>Best current contact information</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="n"/>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>What they already know</t>
+        </is>
+      </c>
+      <c r="F22" s="20" t="n"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="24" t="inlineStr"/>
+      <c r="B23" s="24" t="inlineStr"/>
+      <c r="C23" s="24" t="inlineStr"/>
+      <c r="D23" s="20" t="n"/>
+      <c r="E23" s="24" t="inlineStr"/>
+      <c r="F23" s="20" t="n"/>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="24" t="inlineStr"/>
+      <c r="B24" s="24" t="inlineStr"/>
+      <c r="C24" s="24" t="inlineStr"/>
+      <c r="D24" s="20" t="n"/>
+      <c r="E24" s="24" t="inlineStr"/>
+      <c r="F24" s="20" t="n"/>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="24" t="inlineStr"/>
+      <c r="B25" s="24" t="inlineStr"/>
+      <c r="C25" s="24" t="inlineStr"/>
+      <c r="D25" s="20" t="n"/>
+      <c r="E25" s="24" t="inlineStr"/>
+      <c r="F25" s="20" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="n"/>
+      <c r="B26" s="21" t="n"/>
+      <c r="C26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="21" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="24">
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E23:F23"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="B9:F9"/>
     <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B16:F16"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="E25:F25"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="E22:F22"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -690,189 +937,164 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Household Handoff Map</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Use one line per area. Delete what does not apply; add your own. This is orientation, not an inventory of every record.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
+      <c r="D1" s="20" t="n"/>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Use this as the index. Do not repeat open-loop or recurring details here; those have their own sheets.</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="20" t="n"/>
+    </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>What exists / what matters</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>Who matters</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>Where the real information lives</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>What is happening now</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>What needs to keep happening</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="72" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+    </row>
+    <row r="5" ht="62" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Home / property</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n"/>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
-    </row>
-    <row r="6" ht="72" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr"/>
+      <c r="C5" s="24" t="inlineStr"/>
+      <c r="D5" s="24" t="inlineStr"/>
+    </row>
+    <row r="6" ht="62" customHeight="1">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>Insurance / claims</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
-    </row>
-    <row r="7" ht="72" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr"/>
+      <c r="C6" s="24" t="inlineStr"/>
+      <c r="D6" s="24" t="inlineStr"/>
+    </row>
+    <row r="7" ht="62" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Money / accounts / bills</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-    </row>
-    <row r="8" ht="72" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr"/>
+      <c r="C7" s="24" t="inlineStr"/>
+      <c r="D7" s="24" t="inlineStr"/>
+    </row>
+    <row r="8" ht="62" customHeight="1">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Health / care</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="72" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr"/>
+      <c r="C8" s="24" t="inlineStr"/>
+      <c r="D8" s="24" t="inlineStr"/>
+    </row>
+    <row r="9" ht="62" customHeight="1">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Identity / legal</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-    </row>
-    <row r="10" ht="72" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr"/>
+      <c r="C9" s="24" t="inlineStr"/>
+      <c r="D9" s="24" t="inlineStr"/>
+    </row>
+    <row r="10" ht="62" customHeight="1">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Children / dependants</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-    </row>
-    <row r="11" ht="72" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr"/>
+      <c r="C10" s="24" t="inlineStr"/>
+      <c r="D10" s="24" t="inlineStr"/>
+    </row>
+    <row r="11" ht="62" customHeight="1">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>Pets</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-    </row>
-    <row r="12" ht="72" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr"/>
+      <c r="C11" s="24" t="inlineStr"/>
+      <c r="D11" s="24" t="inlineStr"/>
+    </row>
+    <row r="12" ht="62" customHeight="1">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Vehicles / equipment</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
-    </row>
-    <row r="13" ht="72" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr"/>
+      <c r="C12" s="24" t="inlineStr"/>
+      <c r="D12" s="24" t="inlineStr"/>
+    </row>
+    <row r="13" ht="62" customHeight="1">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>Digital services / devices</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
-    </row>
-    <row r="14" ht="72" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr"/>
+      <c r="C13" s="24" t="inlineStr"/>
+      <c r="D13" s="24" t="inlineStr"/>
+    </row>
+    <row r="14" ht="62" customHeight="1">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
+      <c r="B14" s="24" t="inlineStr"/>
+      <c r="C14" s="24" t="inlineStr"/>
+      <c r="D14" s="24" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F14"/>
+  <autoFilter ref="A4:D14"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -910,7 +1132,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -934,7 +1155,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>When to check / deadline</t>
+          <t>Next check / deadline</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -1088,7 +1309,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -1107,7 +1327,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Where the governing information lives</t>
+          <t>Where the real information lives</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1237,12 +1457,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1250,18 +1470,17 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Protected Access</t>
+          <t>Authority &amp; Access</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Record where access, recovery, emergency-access, legacy, or delegation arrangements are managed. Never record the secret itself.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Point to where authority or protected access is managed. Record arrangements, not secrets; use this sheet as pointers, not replacements.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -1275,12 +1494,12 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Emergency / legacy / delegation arrangement</t>
+          <t>What arrangement is set up</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Who knows the arrangement exists</t>
+          <t>Who knows it exists</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1354,46 +1573,147 @@
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="9" t="n"/>
     </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Do not store here:</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>Passwords, PINs, recovery codes, encryption keys, banking credentials, security answers, or other secrets.</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="20" t="n"/>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
+      <c r="A13" s="17" t="inlineStr"/>
+      <c r="B13" s="17" t="inlineStr"/>
+      <c r="C13" s="17" t="inlineStr"/>
+      <c r="D13" s="17" t="inlineStr"/>
+      <c r="E13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-    </row>
-    <row r="15"/>
-    <row r="16"/>
+      <c r="A14" s="17" t="inlineStr"/>
+      <c r="B14" s="17" t="inlineStr"/>
+      <c r="C14" s="17" t="inlineStr"/>
+      <c r="D14" s="17" t="inlineStr"/>
+      <c r="E14" s="17" t="inlineStr"/>
+    </row>
+    <row r="15" ht="25" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Governing Documents &amp; Professional Contacts</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="20" t="n"/>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>This section is a pointer only. The document, institution, account mechanism, or formal process remains the source to rely on.</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="n"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="20" t="n"/>
+    </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>Do not store here:</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Passwords, PINs, recovery codes, encryption keys, banking credentials, security answers, or other secrets.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A17" s="17" t="inlineStr"/>
+      <c r="B17" s="17" t="inlineStr"/>
+      <c r="C17" s="17" t="inlineStr"/>
+      <c r="D17" s="17" t="inlineStr"/>
+      <c r="E17" s="17" t="inlineStr"/>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>Document / arrangement</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Where the current version lives</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>Professional / institution</t>
+        </is>
+      </c>
+      <c r="D18" s="22" t="inlineStr">
+        <is>
+          <t>Who should know it exists</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>Last checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>Will / estate documents, if applicable</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="inlineStr"/>
+      <c r="C19" s="24" t="inlineStr"/>
+      <c r="D19" s="24" t="inlineStr"/>
+      <c r="E19" s="24" t="inlineStr"/>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Power of attorney / personal directive / similar, if applicable</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="inlineStr"/>
+      <c r="C20" s="24" t="inlineStr"/>
+      <c r="D20" s="24" t="inlineStr"/>
+      <c r="E20" s="24" t="inlineStr"/>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Beneficiary / account arrangements, if applicable</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr"/>
+      <c r="C21" s="24" t="inlineStr"/>
+      <c r="D21" s="24" t="inlineStr"/>
+      <c r="E21" s="24" t="inlineStr"/>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr"/>
+      <c r="C22" s="24" t="inlineStr"/>
+      <c r="D22" s="24" t="inlineStr"/>
+      <c r="E22" s="24" t="inlineStr"/>
+    </row>
+    <row r="23" ht="34" customHeight="1"/>
+    <row r="24" ht="48" customHeight="1"/>
+    <row r="25" ht="48" customHeight="1"/>
+    <row r="26" ht="48" customHeight="1"/>
+    <row r="27" ht="48" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A4:E14"/>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
@@ -1431,7 +1751,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -1505,8 +1824,6 @@
       <c r="B10" s="13" t="n"/>
       <c r="C10" s="9" t="n"/>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
@@ -1601,7 +1918,7 @@
     <row r="21" ht="34" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Periodic check for quiet changes in recurring responsibilities or access arrangements</t>
+          <t>Periodic check for quiet changes in recurring responsibilities, open loops, or access arrangements</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -1610,8 +1927,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>

</xml_diff>